<commit_message>
Add Comment In Code
</commit_message>
<xml_diff>
--- a/SeleniumTests/Import Transaction/With Data/b2c_invoice_template.xlsx
+++ b/SeleniumTests/Import Transaction/With Data/b2c_invoice_template.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="29328"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="29426"/>
   <workbookPr codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\e-invoice\SeleniumTests\Import Transaction\With Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F54548A2-84D3-4271-B2B5-EA2F62FCA70C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{00B3F52D-B25E-46DD-A3F7-D45A7B4B9594}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="36630" yWindow="5040" windowWidth="17280" windowHeight="9960" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Transaction" sheetId="1" r:id="rId1"/>
@@ -467,10 +467,10 @@
     <t>2.00</t>
   </si>
   <si>
-    <t>B2CINV1011_000035</t>
-  </si>
-  <si>
-    <t>B2CINV1011_000036</t>
+    <t>B2CINV1216_000002</t>
+  </si>
+  <si>
+    <t>B2CINV1216_000001</t>
   </si>
 </sst>
 </file>
@@ -1514,7 +1514,7 @@
         <v>132</v>
       </c>
       <c r="D4" s="2" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="E4" s="2" t="s">
         <v>133</v>
@@ -1661,7 +1661,7 @@
         <v>132</v>
       </c>
       <c r="D5" s="2" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="E5" s="2" t="s">
         <v>133</v>

</xml_diff>